<commit_message>
update on june plan
</commit_message>
<xml_diff>
--- a/sales_app/data/Full Plan workflow.xlsx
+++ b/sales_app/data/Full Plan workflow.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/macintoshi/Desktop/Django_unchainded/sales_app/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{461E3C71-400D-274A-9514-6E60FB1D7EDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9539B18C-FEA1-2B48-BC8A-C75BC45CFA76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="22020" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1042" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1081" uniqueCount="78">
   <si>
     <t>location</t>
   </si>
@@ -6405,7 +6405,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{650603AD-9288-4A14-8188-833FDDD6C46C}">
-  <dimension ref="A1:K413"/>
+  <dimension ref="A1:K426"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="21.1640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="5" max="7" width="21.1640625" style="24"/>
@@ -15634,6 +15634,227 @@
         <v>51</v>
       </c>
       <c r="E413" s="33">
+        <v>16000</v>
+      </c>
+    </row>
+    <row r="414" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A414">
+        <v>2026</v>
+      </c>
+      <c r="B414">
+        <v>6</v>
+      </c>
+      <c r="C414" t="s">
+        <v>1</v>
+      </c>
+      <c r="D414" t="s">
+        <v>62</v>
+      </c>
+      <c r="E414" s="33">
+        <v>113000</v>
+      </c>
+    </row>
+    <row r="415" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A415">
+        <v>2026</v>
+      </c>
+      <c r="B415">
+        <v>6</v>
+      </c>
+      <c r="C415" t="s">
+        <v>2</v>
+      </c>
+      <c r="D415" t="s">
+        <v>55</v>
+      </c>
+      <c r="E415" s="33">
+        <v>82000</v>
+      </c>
+    </row>
+    <row r="416" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A416">
+        <v>2026</v>
+      </c>
+      <c r="B416">
+        <v>6</v>
+      </c>
+      <c r="C416" t="s">
+        <v>3</v>
+      </c>
+      <c r="D416" t="s">
+        <v>48</v>
+      </c>
+      <c r="E416" s="33">
+        <v>58000</v>
+      </c>
+    </row>
+    <row r="417" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A417">
+        <v>2026</v>
+      </c>
+      <c r="B417">
+        <v>6</v>
+      </c>
+      <c r="C417" t="s">
+        <v>4</v>
+      </c>
+      <c r="D417" t="s">
+        <v>63</v>
+      </c>
+      <c r="E417" s="33">
+        <v>55000</v>
+      </c>
+    </row>
+    <row r="418" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A418">
+        <v>2026</v>
+      </c>
+      <c r="B418">
+        <v>6</v>
+      </c>
+      <c r="C418" t="s">
+        <v>5</v>
+      </c>
+      <c r="D418" t="s">
+        <v>54</v>
+      </c>
+      <c r="E418" s="33">
+        <v>57000</v>
+      </c>
+    </row>
+    <row r="419" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A419">
+        <v>2026</v>
+      </c>
+      <c r="B419">
+        <v>6</v>
+      </c>
+      <c r="C419" t="s">
+        <v>6</v>
+      </c>
+      <c r="D419" t="s">
+        <v>57</v>
+      </c>
+      <c r="E419" s="33">
+        <v>33000</v>
+      </c>
+    </row>
+    <row r="420" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A420">
+        <v>2026</v>
+      </c>
+      <c r="B420">
+        <v>6</v>
+      </c>
+      <c r="C420" t="s">
+        <v>7</v>
+      </c>
+      <c r="D420" t="s">
+        <v>64</v>
+      </c>
+      <c r="E420" s="33">
+        <v>43000</v>
+      </c>
+    </row>
+    <row r="421" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A421">
+        <v>2026</v>
+      </c>
+      <c r="B421">
+        <v>6</v>
+      </c>
+      <c r="C421" t="s">
+        <v>8</v>
+      </c>
+      <c r="D421" t="s">
+        <v>58</v>
+      </c>
+      <c r="E421" s="33">
+        <v>45000</v>
+      </c>
+    </row>
+    <row r="422" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A422">
+        <v>2026</v>
+      </c>
+      <c r="B422">
+        <v>6</v>
+      </c>
+      <c r="C422" t="s">
+        <v>9</v>
+      </c>
+      <c r="D422" t="s">
+        <v>49</v>
+      </c>
+      <c r="E422" s="33">
+        <v>31000</v>
+      </c>
+    </row>
+    <row r="423" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A423">
+        <v>2026</v>
+      </c>
+      <c r="B423">
+        <v>6</v>
+      </c>
+      <c r="C423" t="s">
+        <v>10</v>
+      </c>
+      <c r="D423" t="s">
+        <v>50</v>
+      </c>
+      <c r="E423" s="33">
+        <v>46000</v>
+      </c>
+    </row>
+    <row r="424" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A424">
+        <v>2026</v>
+      </c>
+      <c r="B424">
+        <v>6</v>
+      </c>
+      <c r="C424" t="s">
+        <v>11</v>
+      </c>
+      <c r="D424" t="s">
+        <v>59</v>
+      </c>
+      <c r="E424" s="33">
+        <v>43000</v>
+      </c>
+    </row>
+    <row r="425" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A425">
+        <v>2026</v>
+      </c>
+      <c r="B425">
+        <v>6</v>
+      </c>
+      <c r="C425" t="s">
+        <v>12</v>
+      </c>
+      <c r="D425" t="s">
+        <v>60</v>
+      </c>
+      <c r="E425" s="33">
+        <v>58000</v>
+      </c>
+    </row>
+    <row r="426" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A426">
+        <v>2026</v>
+      </c>
+      <c r="B426">
+        <v>6</v>
+      </c>
+      <c r="C426" t="s">
+        <v>13</v>
+      </c>
+      <c r="D426" t="s">
+        <v>51</v>
+      </c>
+      <c r="E426" s="33">
         <v>16000</v>
       </c>
     </row>
@@ -15891,7 +16112,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51FCE611-90D9-BD45-9A96-E3469C310DDF}">
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:C29"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="21.5" bestFit="1" customWidth="1"/>
@@ -16015,6 +16236,149 @@
         <v>761000</v>
       </c>
     </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A17" s="33" t="s">
+        <v>65</v>
+      </c>
+      <c r="B17" s="33">
+        <v>113000</v>
+      </c>
+      <c r="C17" s="33">
+        <v>96050</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A18" s="33" t="s">
+        <v>66</v>
+      </c>
+      <c r="B18" s="33">
+        <v>82000</v>
+      </c>
+      <c r="C18" s="33">
+        <v>69700</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A19" s="33" t="s">
+        <v>67</v>
+      </c>
+      <c r="B19" s="33">
+        <v>58000</v>
+      </c>
+      <c r="C19" s="33">
+        <v>49300</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A20" s="33" t="s">
+        <v>68</v>
+      </c>
+      <c r="B20" s="33">
+        <v>55000</v>
+      </c>
+      <c r="C20" s="33">
+        <v>46750</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A21" s="33" t="s">
+        <v>69</v>
+      </c>
+      <c r="B21" s="33">
+        <v>57000</v>
+      </c>
+      <c r="C21" s="33">
+        <v>48450</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A22" s="33" t="s">
+        <v>70</v>
+      </c>
+      <c r="B22" s="33">
+        <v>33000</v>
+      </c>
+      <c r="C22" s="33">
+        <v>28050</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A23" s="33" t="s">
+        <v>71</v>
+      </c>
+      <c r="B23" s="33">
+        <v>43000</v>
+      </c>
+      <c r="C23" s="33">
+        <v>36550</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A24" s="33" t="s">
+        <v>72</v>
+      </c>
+      <c r="B24" s="33">
+        <v>45000</v>
+      </c>
+      <c r="C24" s="33">
+        <v>38250</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A25" s="33" t="s">
+        <v>73</v>
+      </c>
+      <c r="B25" s="33">
+        <v>31000</v>
+      </c>
+      <c r="C25" s="33">
+        <v>26350</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A26" s="33" t="s">
+        <v>74</v>
+      </c>
+      <c r="B26" s="33">
+        <v>46000</v>
+      </c>
+      <c r="C26" s="33">
+        <v>39100</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A27" s="33" t="s">
+        <v>75</v>
+      </c>
+      <c r="B27" s="33">
+        <v>43000</v>
+      </c>
+      <c r="C27" s="33">
+        <v>36550</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A28" s="33" t="s">
+        <v>76</v>
+      </c>
+      <c r="B28" s="33">
+        <v>58000</v>
+      </c>
+      <c r="C28" s="33">
+        <v>49300</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A29" s="33" t="s">
+        <v>77</v>
+      </c>
+      <c r="B29" s="33">
+        <v>16000</v>
+      </c>
+      <c r="C29" s="33">
+        <v>13600</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
update on august plan
</commit_message>
<xml_diff>
--- a/sales_app/data/Full Plan workflow.xlsx
+++ b/sales_app/data/Full Plan workflow.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/macintoshi/Desktop/Django_unchainded/sales_app/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41DA545B-8933-0242-ABBD-D5727205F2D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0A433AB-DA61-FF47-A28A-2B69947EC19F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="22020" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1134" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1172" uniqueCount="79">
   <si>
     <t>location</t>
   </si>
@@ -582,8 +582,8 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="9" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="9" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -6446,7 +6446,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{650603AD-9288-4A14-8188-833FDDD6C46C}">
-  <dimension ref="A1:K439"/>
+  <dimension ref="A1:K452"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="21.1640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="5" max="7" width="21.1640625" style="24"/>
@@ -16117,6 +16117,227 @@
         <v>51</v>
       </c>
       <c r="E439" s="24">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="440" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A440">
+        <v>2026</v>
+      </c>
+      <c r="B440">
+        <v>8</v>
+      </c>
+      <c r="C440" t="s">
+        <v>1</v>
+      </c>
+      <c r="D440" t="s">
+        <v>62</v>
+      </c>
+      <c r="E440" s="24">
+        <v>123000</v>
+      </c>
+    </row>
+    <row r="441" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A441">
+        <v>2026</v>
+      </c>
+      <c r="B441">
+        <v>8</v>
+      </c>
+      <c r="C441" t="s">
+        <v>2</v>
+      </c>
+      <c r="D441" t="s">
+        <v>55</v>
+      </c>
+      <c r="E441" s="24">
+        <v>103000</v>
+      </c>
+    </row>
+    <row r="442" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A442">
+        <v>2026</v>
+      </c>
+      <c r="B442">
+        <v>8</v>
+      </c>
+      <c r="C442" t="s">
+        <v>3</v>
+      </c>
+      <c r="D442" t="s">
+        <v>48</v>
+      </c>
+      <c r="E442" s="24">
+        <v>62000</v>
+      </c>
+    </row>
+    <row r="443" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A443">
+        <v>2026</v>
+      </c>
+      <c r="B443">
+        <v>8</v>
+      </c>
+      <c r="C443" t="s">
+        <v>4</v>
+      </c>
+      <c r="D443" t="s">
+        <v>63</v>
+      </c>
+      <c r="E443" s="24">
+        <v>60000</v>
+      </c>
+    </row>
+    <row r="444" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A444">
+        <v>2026</v>
+      </c>
+      <c r="B444">
+        <v>8</v>
+      </c>
+      <c r="C444" t="s">
+        <v>5</v>
+      </c>
+      <c r="D444" t="s">
+        <v>54</v>
+      </c>
+      <c r="E444" s="24">
+        <v>70000</v>
+      </c>
+    </row>
+    <row r="445" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A445">
+        <v>2026</v>
+      </c>
+      <c r="B445">
+        <v>8</v>
+      </c>
+      <c r="C445" t="s">
+        <v>6</v>
+      </c>
+      <c r="D445" t="s">
+        <v>57</v>
+      </c>
+      <c r="E445" s="24">
+        <v>45000</v>
+      </c>
+    </row>
+    <row r="446" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A446">
+        <v>2026</v>
+      </c>
+      <c r="B446">
+        <v>8</v>
+      </c>
+      <c r="C446" t="s">
+        <v>7</v>
+      </c>
+      <c r="D446" t="s">
+        <v>64</v>
+      </c>
+      <c r="E446" s="24">
+        <v>43000</v>
+      </c>
+    </row>
+    <row r="447" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A447">
+        <v>2026</v>
+      </c>
+      <c r="B447">
+        <v>8</v>
+      </c>
+      <c r="C447" t="s">
+        <v>8</v>
+      </c>
+      <c r="D447" t="s">
+        <v>58</v>
+      </c>
+      <c r="E447" s="24">
+        <v>65000</v>
+      </c>
+    </row>
+    <row r="448" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A448">
+        <v>2026</v>
+      </c>
+      <c r="B448">
+        <v>8</v>
+      </c>
+      <c r="C448" t="s">
+        <v>9</v>
+      </c>
+      <c r="D448" t="s">
+        <v>49</v>
+      </c>
+      <c r="E448" s="24">
+        <v>35000</v>
+      </c>
+    </row>
+    <row r="449" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A449">
+        <v>2026</v>
+      </c>
+      <c r="B449">
+        <v>8</v>
+      </c>
+      <c r="C449" t="s">
+        <v>10</v>
+      </c>
+      <c r="D449" t="s">
+        <v>50</v>
+      </c>
+      <c r="E449" s="24">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="450" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A450">
+        <v>2026</v>
+      </c>
+      <c r="B450">
+        <v>8</v>
+      </c>
+      <c r="C450" t="s">
+        <v>11</v>
+      </c>
+      <c r="D450" t="s">
+        <v>59</v>
+      </c>
+      <c r="E450" s="24">
+        <v>43000</v>
+      </c>
+    </row>
+    <row r="451" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A451">
+        <v>2026</v>
+      </c>
+      <c r="B451">
+        <v>8</v>
+      </c>
+      <c r="C451" t="s">
+        <v>12</v>
+      </c>
+      <c r="D451" t="s">
+        <v>60</v>
+      </c>
+      <c r="E451" s="24">
+        <v>108000</v>
+      </c>
+    </row>
+    <row r="452" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A452">
+        <v>2026</v>
+      </c>
+      <c r="B452">
+        <v>8</v>
+      </c>
+      <c r="C452" t="s">
+        <v>13</v>
+      </c>
+      <c r="D452" t="s">
+        <v>51</v>
+      </c>
+      <c r="E452" s="24">
         <v>20000</v>
       </c>
     </row>
@@ -16374,14 +16595,15 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51FCE611-90D9-BD45-9A96-E3469C310DDF}">
-  <dimension ref="A1:I29"/>
+  <dimension ref="A1:P29"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="21.5" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="20.33203125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="18.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="21" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:16" ht="21" x14ac:dyDescent="0.25">
       <c r="A1" s="28" t="s">
         <v>65</v>
       </c>
@@ -16398,7 +16620,7 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A2" s="28" t="s">
         <v>66</v>
       </c>
@@ -16418,7 +16640,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A3" s="28" t="s">
         <v>67</v>
       </c>
@@ -16437,8 +16659,14 @@
       <c r="I3" s="38" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="L3" s="33"/>
+      <c r="M3" s="33">
+        <v>123000</v>
+      </c>
+      <c r="N3" s="33"/>
+      <c r="O3" s="33"/>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A4" s="28" t="s">
         <v>68</v>
       </c>
@@ -16457,8 +16685,17 @@
       <c r="I4" s="39" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="L4" s="33" t="s">
+        <v>66</v>
+      </c>
+      <c r="M4" s="33">
+        <v>103000</v>
+      </c>
+      <c r="N4" s="33"/>
+      <c r="O4" s="33"/>
+      <c r="P4" s="33"/>
+    </row>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A5" s="28" t="s">
         <v>69</v>
       </c>
@@ -16477,8 +16714,17 @@
       <c r="I5" s="38" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="L5" s="33" t="s">
+        <v>67</v>
+      </c>
+      <c r="M5" s="33">
+        <v>62000</v>
+      </c>
+      <c r="N5" s="33"/>
+      <c r="O5" s="33"/>
+      <c r="P5" s="33"/>
+    </row>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A6" s="28" t="s">
         <v>70</v>
       </c>
@@ -16497,8 +16743,17 @@
       <c r="I6" s="39" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="L6" s="33" t="s">
+        <v>68</v>
+      </c>
+      <c r="M6" s="33">
+        <v>60000</v>
+      </c>
+      <c r="N6" s="33"/>
+      <c r="O6" s="33"/>
+      <c r="P6" s="33"/>
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A7" s="28" t="s">
         <v>71</v>
       </c>
@@ -16517,8 +16772,17 @@
       <c r="I7" s="38" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="L7" s="33" t="s">
+        <v>69</v>
+      </c>
+      <c r="M7" s="33">
+        <v>70000</v>
+      </c>
+      <c r="N7" s="33"/>
+      <c r="O7" s="33"/>
+      <c r="P7" s="33"/>
+    </row>
+    <row r="8" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A8" s="28" t="s">
         <v>72</v>
       </c>
@@ -16537,8 +16801,17 @@
       <c r="I8" s="39" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="L8" s="33" t="s">
+        <v>70</v>
+      </c>
+      <c r="M8" s="33">
+        <v>45000</v>
+      </c>
+      <c r="N8" s="33"/>
+      <c r="O8" s="33"/>
+      <c r="P8" s="33"/>
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A9" s="28" t="s">
         <v>73</v>
       </c>
@@ -16557,8 +16830,17 @@
       <c r="I9" s="38" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="L9" s="33" t="s">
+        <v>71</v>
+      </c>
+      <c r="M9" s="33">
+        <v>43000</v>
+      </c>
+      <c r="N9" s="33"/>
+      <c r="O9" s="33"/>
+      <c r="P9" s="33"/>
+    </row>
+    <row r="10" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A10" s="28" t="s">
         <v>74</v>
       </c>
@@ -16577,8 +16859,17 @@
       <c r="I10" s="39" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="L10" s="33" t="s">
+        <v>72</v>
+      </c>
+      <c r="M10" s="33">
+        <v>65000</v>
+      </c>
+      <c r="N10" s="33"/>
+      <c r="O10" s="33"/>
+      <c r="P10" s="33"/>
+    </row>
+    <row r="11" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A11" s="28" t="s">
         <v>75</v>
       </c>
@@ -16597,8 +16888,17 @@
       <c r="I11" s="38" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="L11" s="33" t="s">
+        <v>73</v>
+      </c>
+      <c r="M11" s="33">
+        <v>35000</v>
+      </c>
+      <c r="N11" s="33"/>
+      <c r="O11" s="33"/>
+      <c r="P11" s="33"/>
+    </row>
+    <row r="12" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A12" s="28" t="s">
         <v>76</v>
       </c>
@@ -16617,8 +16917,17 @@
       <c r="I12" s="39" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="L12" s="33" t="s">
+        <v>74</v>
+      </c>
+      <c r="M12" s="33">
+        <v>50000</v>
+      </c>
+      <c r="N12" s="33"/>
+      <c r="O12" s="33"/>
+      <c r="P12" s="33"/>
+    </row>
+    <row r="13" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A13" s="28" t="s">
         <v>77</v>
       </c>
@@ -16637,8 +16946,17 @@
       <c r="I13" s="38" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="L13" s="33" t="s">
+        <v>75</v>
+      </c>
+      <c r="M13" s="33">
+        <v>43000</v>
+      </c>
+      <c r="N13" s="33"/>
+      <c r="O13" s="33"/>
+      <c r="P13" s="33"/>
+    </row>
+    <row r="14" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A14" s="28" t="s">
         <v>14</v>
       </c>
@@ -16657,8 +16975,17 @@
       <c r="I14" s="39" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="15" spans="1:9" ht="22" x14ac:dyDescent="0.3">
+      <c r="L14" s="33" t="s">
+        <v>76</v>
+      </c>
+      <c r="M14" s="33">
+        <v>108000</v>
+      </c>
+      <c r="N14" s="33"/>
+      <c r="O14" s="33"/>
+      <c r="P14" s="33"/>
+    </row>
+    <row r="15" spans="1:16" ht="22" x14ac:dyDescent="0.3">
       <c r="A15" s="29"/>
       <c r="B15" s="30">
         <v>761000</v>
@@ -16670,6 +16997,15 @@
       <c r="H15" s="33">
         <v>735250</v>
       </c>
+      <c r="L15" s="33" t="s">
+        <v>77</v>
+      </c>
+      <c r="M15" s="33">
+        <v>20000</v>
+      </c>
+      <c r="N15" s="33"/>
+      <c r="O15" s="33"/>
+      <c r="P15" s="33"/>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A17" s="33" t="s">

</xml_diff>

<commit_message>
update on plan workflow
</commit_message>
<xml_diff>
--- a/sales_app/data/Full Plan workflow.xlsx
+++ b/sales_app/data/Full Plan workflow.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/macintoshi/Desktop/Django_unchainded/sales_app/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0A433AB-DA61-FF47-A28A-2B69947EC19F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{204CE33A-E92A-0B41-9426-8FC9E3DA11E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="22020" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1172" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1170" uniqueCount="79">
   <si>
     <t>location</t>
   </si>
@@ -2365,8 +2365,8 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{1B929C5C-00E3-4412-8552-8FA882683BA9}" name="Table7" displayName="Table7" ref="A1:G1048575" totalsRowShown="0">
-  <autoFilter ref="A1:G1048575" xr:uid="{1B929C5C-00E3-4412-8552-8FA882683BA9}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{1B929C5C-00E3-4412-8552-8FA882683BA9}" name="Table7" displayName="Table7" ref="A1:G1048574" totalsRowShown="0">
+  <autoFilter ref="A1:G1048574" xr:uid="{1B929C5C-00E3-4412-8552-8FA882683BA9}"/>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{1EBC0AF8-CA34-45C1-AB80-32D4A4F106A0}" name="Year"/>
     <tableColumn id="2" xr3:uid="{3A8A3FA9-4717-4E43-B5C4-95DC6B0AD9C5}" name="Month"/>
@@ -6446,7 +6446,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{650603AD-9288-4A14-8188-833FDDD6C46C}">
-  <dimension ref="A1:K452"/>
+  <dimension ref="A1:K451"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="21.1640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="5" max="7" width="21.1640625" style="24"/>
@@ -16322,23 +16322,6 @@
       </c>
       <c r="E451" s="24">
         <v>108000</v>
-      </c>
-    </row>
-    <row r="452" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A452">
-        <v>2026</v>
-      </c>
-      <c r="B452">
-        <v>8</v>
-      </c>
-      <c r="C452" t="s">
-        <v>13</v>
-      </c>
-      <c r="D452" t="s">
-        <v>51</v>
-      </c>
-      <c r="E452" s="24">
-        <v>20000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update on plan september
</commit_message>
<xml_diff>
--- a/sales_app/data/Full Plan workflow.xlsx
+++ b/sales_app/data/Full Plan workflow.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/macintoshi/Desktop/Django_unchainded/sales_app/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{204CE33A-E92A-0B41-9426-8FC9E3DA11E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF7C06D8-5BE5-D542-8105-1C869EE4F491}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="22020" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1170" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1210" uniqueCount="93">
   <si>
     <t>location</t>
   </si>
@@ -280,12 +280,280 @@
   <si>
     <t>july</t>
   </si>
+  <si>
+    <t>სექტემბერი</t>
+  </si>
+  <si>
+    <t>ობიექტი</t>
+  </si>
+  <si>
+    <r>
+      <t>გეგმა</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t> 100%</t>
+    </r>
+  </si>
+  <si>
+    <t>ვაკე</t>
+  </si>
+  <si>
+    <r>
+      <t>ისტ</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t> </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>პოინტი</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>სითი</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t> </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>მოლი</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t> </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>გლდანი</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>გლდანი</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t> </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>მოლი</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>სითი</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t> </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>მოლისაბურთალო</t>
+    </r>
+  </si>
+  <si>
+    <t>პეკინი</t>
+  </si>
+  <si>
+    <r>
+      <t>ბათუმი</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t> </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>გრანდ</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t> </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>მოლი</t>
+    </r>
+  </si>
+  <si>
+    <t>პლეხანოვი</t>
+  </si>
+  <si>
+    <r>
+      <t>გუდვილი</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t> </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>დიღომი</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>ბათუმი</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t> </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>მეტრო</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t> </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>მოლი</t>
+    </r>
+  </si>
+  <si>
+    <t>ჯამი</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="13" x14ac:knownFonts="1">
+  <fonts count="17" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -374,6 +642,34 @@
       <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF1F1F1F"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF1F1F1F"/>
+      <name val="Arial"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -525,7 +821,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -587,6 +883,10 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="9" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="3" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -6446,7 +6746,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{650603AD-9288-4A14-8188-833FDDD6C46C}">
-  <dimension ref="A1:K451"/>
+  <dimension ref="A1:K463"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="21.1640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="5" max="7" width="21.1640625" style="24"/>
@@ -16322,6 +16622,210 @@
       </c>
       <c r="E451" s="24">
         <v>108000</v>
+      </c>
+    </row>
+    <row r="452" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A452">
+        <v>2026</v>
+      </c>
+      <c r="B452">
+        <v>9</v>
+      </c>
+      <c r="C452" t="s">
+        <v>1</v>
+      </c>
+      <c r="D452" t="s">
+        <v>62</v>
+      </c>
+      <c r="E452">
+        <v>121000</v>
+      </c>
+    </row>
+    <row r="453" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A453">
+        <v>2026</v>
+      </c>
+      <c r="B453">
+        <v>9</v>
+      </c>
+      <c r="C453" t="s">
+        <v>2</v>
+      </c>
+      <c r="D453" t="s">
+        <v>55</v>
+      </c>
+      <c r="E453">
+        <v>87000</v>
+      </c>
+    </row>
+    <row r="454" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A454">
+        <v>2026</v>
+      </c>
+      <c r="B454">
+        <v>9</v>
+      </c>
+      <c r="C454" t="s">
+        <v>3</v>
+      </c>
+      <c r="D454" t="s">
+        <v>48</v>
+      </c>
+      <c r="E454">
+        <v>57000</v>
+      </c>
+    </row>
+    <row r="455" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A455">
+        <v>2026</v>
+      </c>
+      <c r="B455">
+        <v>9</v>
+      </c>
+      <c r="C455" t="s">
+        <v>4</v>
+      </c>
+      <c r="D455" t="s">
+        <v>63</v>
+      </c>
+      <c r="E455">
+        <v>55000</v>
+      </c>
+    </row>
+    <row r="456" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A456">
+        <v>2026</v>
+      </c>
+      <c r="B456">
+        <v>9</v>
+      </c>
+      <c r="C456" t="s">
+        <v>5</v>
+      </c>
+      <c r="D456" t="s">
+        <v>54</v>
+      </c>
+      <c r="E456">
+        <v>67000</v>
+      </c>
+    </row>
+    <row r="457" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A457">
+        <v>2026</v>
+      </c>
+      <c r="B457">
+        <v>9</v>
+      </c>
+      <c r="C457" t="s">
+        <v>6</v>
+      </c>
+      <c r="D457" t="s">
+        <v>57</v>
+      </c>
+      <c r="E457">
+        <v>44000</v>
+      </c>
+    </row>
+    <row r="458" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A458">
+        <v>2026</v>
+      </c>
+      <c r="B458">
+        <v>9</v>
+      </c>
+      <c r="C458" t="s">
+        <v>7</v>
+      </c>
+      <c r="D458" t="s">
+        <v>64</v>
+      </c>
+      <c r="E458">
+        <v>42000</v>
+      </c>
+    </row>
+    <row r="459" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A459">
+        <v>2026</v>
+      </c>
+      <c r="B459">
+        <v>9</v>
+      </c>
+      <c r="C459" t="s">
+        <v>8</v>
+      </c>
+      <c r="D459" t="s">
+        <v>58</v>
+      </c>
+      <c r="E459">
+        <v>48000</v>
+      </c>
+    </row>
+    <row r="460" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A460">
+        <v>2026</v>
+      </c>
+      <c r="B460">
+        <v>9</v>
+      </c>
+      <c r="C460" t="s">
+        <v>9</v>
+      </c>
+      <c r="D460" t="s">
+        <v>49</v>
+      </c>
+      <c r="E460">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="461" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A461">
+        <v>2026</v>
+      </c>
+      <c r="B461">
+        <v>9</v>
+      </c>
+      <c r="C461" t="s">
+        <v>10</v>
+      </c>
+      <c r="D461" t="s">
+        <v>50</v>
+      </c>
+      <c r="E461">
+        <v>45000</v>
+      </c>
+    </row>
+    <row r="462" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A462">
+        <v>2026</v>
+      </c>
+      <c r="B462">
+        <v>9</v>
+      </c>
+      <c r="C462" t="s">
+        <v>11</v>
+      </c>
+      <c r="D462" t="s">
+        <v>59</v>
+      </c>
+      <c r="E462">
+        <v>46000</v>
+      </c>
+    </row>
+    <row r="463" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A463">
+        <v>2026</v>
+      </c>
+      <c r="B463">
+        <v>9</v>
+      </c>
+      <c r="C463" t="s">
+        <v>12</v>
+      </c>
+      <c r="D463" t="s">
+        <v>60</v>
+      </c>
+      <c r="E463">
+        <v>63000</v>
       </c>
     </row>
   </sheetData>
@@ -16578,15 +17082,16 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51FCE611-90D9-BD45-9A96-E3469C310DDF}">
-  <dimension ref="A1:P29"/>
+  <dimension ref="A1:R29"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="21.5" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="20.33203125" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="18.33203125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="22.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="21" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:18" ht="21" x14ac:dyDescent="0.25">
       <c r="A1" s="28" t="s">
         <v>65</v>
       </c>
@@ -16602,8 +17107,14 @@
       <c r="H1" s="42">
         <v>0.85</v>
       </c>
-    </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q1" s="43">
+        <v>2026</v>
+      </c>
+      <c r="R1" s="44" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A2" s="28" t="s">
         <v>66</v>
       </c>
@@ -16622,8 +17133,14 @@
       <c r="I2" s="39" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q2" s="45" t="s">
+        <v>80</v>
+      </c>
+      <c r="R2" s="45" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A3" s="28" t="s">
         <v>67</v>
       </c>
@@ -16648,8 +17165,14 @@
       </c>
       <c r="N3" s="33"/>
       <c r="O3" s="33"/>
-    </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q3" s="45" t="s">
+        <v>82</v>
+      </c>
+      <c r="R3" s="46">
+        <v>46000</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A4" s="28" t="s">
         <v>68</v>
       </c>
@@ -16677,8 +17200,14 @@
       <c r="N4" s="33"/>
       <c r="O4" s="33"/>
       <c r="P4" s="33"/>
-    </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q4" s="45" t="s">
+        <v>83</v>
+      </c>
+      <c r="R4" s="46">
+        <v>67000</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A5" s="28" t="s">
         <v>69</v>
       </c>
@@ -16706,8 +17235,14 @@
       <c r="N5" s="33"/>
       <c r="O5" s="33"/>
       <c r="P5" s="33"/>
-    </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q5" s="45" t="s">
+        <v>84</v>
+      </c>
+      <c r="R5" s="46">
+        <v>44000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A6" s="28" t="s">
         <v>70</v>
       </c>
@@ -16735,8 +17270,14 @@
       <c r="N6" s="33"/>
       <c r="O6" s="33"/>
       <c r="P6" s="33"/>
-    </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q6" s="45" t="s">
+        <v>85</v>
+      </c>
+      <c r="R6" s="46">
+        <v>57000</v>
+      </c>
+    </row>
+    <row r="7" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A7" s="28" t="s">
         <v>71</v>
       </c>
@@ -16764,8 +17305,14 @@
       <c r="N7" s="33"/>
       <c r="O7" s="33"/>
       <c r="P7" s="33"/>
-    </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q7" s="45" t="s">
+        <v>86</v>
+      </c>
+      <c r="R7" s="46">
+        <v>121000</v>
+      </c>
+    </row>
+    <row r="8" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A8" s="28" t="s">
         <v>72</v>
       </c>
@@ -16793,8 +17340,14 @@
       <c r="N8" s="33"/>
       <c r="O8" s="33"/>
       <c r="P8" s="33"/>
-    </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q8" s="45" t="s">
+        <v>87</v>
+      </c>
+      <c r="R8" s="46">
+        <v>55000</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A9" s="28" t="s">
         <v>73</v>
       </c>
@@ -16822,8 +17375,14 @@
       <c r="N9" s="33"/>
       <c r="O9" s="33"/>
       <c r="P9" s="33"/>
-    </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q9" s="45" t="s">
+        <v>88</v>
+      </c>
+      <c r="R9" s="46">
+        <v>63000</v>
+      </c>
+    </row>
+    <row r="10" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A10" s="28" t="s">
         <v>74</v>
       </c>
@@ -16851,8 +17410,14 @@
       <c r="N10" s="33"/>
       <c r="O10" s="33"/>
       <c r="P10" s="33"/>
-    </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q10" s="45" t="s">
+        <v>89</v>
+      </c>
+      <c r="R10" s="46">
+        <v>42000</v>
+      </c>
+    </row>
+    <row r="11" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A11" s="28" t="s">
         <v>75</v>
       </c>
@@ -16880,8 +17445,14 @@
       <c r="N11" s="33"/>
       <c r="O11" s="33"/>
       <c r="P11" s="33"/>
-    </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q11" s="45" t="s">
+        <v>90</v>
+      </c>
+      <c r="R11" s="46">
+        <v>45000</v>
+      </c>
+    </row>
+    <row r="12" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A12" s="28" t="s">
         <v>76</v>
       </c>
@@ -16909,8 +17480,14 @@
       <c r="N12" s="33"/>
       <c r="O12" s="33"/>
       <c r="P12" s="33"/>
-    </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q12" s="45" t="s">
+        <v>49</v>
+      </c>
+      <c r="R12" s="46">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="13" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A13" s="28" t="s">
         <v>77</v>
       </c>
@@ -16938,8 +17515,14 @@
       <c r="N13" s="33"/>
       <c r="O13" s="33"/>
       <c r="P13" s="33"/>
-    </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q13" s="45" t="s">
+        <v>91</v>
+      </c>
+      <c r="R13" s="46">
+        <v>48000</v>
+      </c>
+    </row>
+    <row r="14" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A14" s="28" t="s">
         <v>14</v>
       </c>
@@ -16967,8 +17550,14 @@
       <c r="N14" s="33"/>
       <c r="O14" s="33"/>
       <c r="P14" s="33"/>
-    </row>
-    <row r="15" spans="1:16" ht="22" x14ac:dyDescent="0.3">
+      <c r="Q14" s="45" t="s">
+        <v>55</v>
+      </c>
+      <c r="R14" s="46">
+        <v>87000</v>
+      </c>
+    </row>
+    <row r="15" spans="1:18" ht="22" x14ac:dyDescent="0.3">
       <c r="A15" s="29"/>
       <c r="B15" s="30">
         <v>761000</v>
@@ -16989,8 +17578,14 @@
       <c r="N15" s="33"/>
       <c r="O15" s="33"/>
       <c r="P15" s="33"/>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="Q15" s="45" t="s">
+        <v>92</v>
+      </c>
+      <c r="R15" s="46">
+        <v>705000</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A17" s="33" t="s">
         <v>65</v>
       </c>
@@ -17000,8 +17595,11 @@
       <c r="C17" s="33">
         <v>96050</v>
       </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D17">
+        <v>121000</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A18" s="33" t="s">
         <v>66</v>
       </c>
@@ -17011,8 +17609,11 @@
       <c r="C18" s="33">
         <v>69700</v>
       </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D18">
+        <v>87000</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A19" s="33" t="s">
         <v>67</v>
       </c>
@@ -17022,8 +17623,11 @@
       <c r="C19" s="33">
         <v>49300</v>
       </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D19">
+        <v>57000</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A20" s="33" t="s">
         <v>68</v>
       </c>
@@ -17033,8 +17637,11 @@
       <c r="C20" s="33">
         <v>46750</v>
       </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D20">
+        <v>55000</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A21" s="33" t="s">
         <v>69</v>
       </c>
@@ -17044,8 +17651,11 @@
       <c r="C21" s="33">
         <v>48450</v>
       </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D21">
+        <v>67000</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A22" s="33" t="s">
         <v>70</v>
       </c>
@@ -17055,8 +17665,11 @@
       <c r="C22" s="33">
         <v>28050</v>
       </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D22">
+        <v>44000</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A23" s="33" t="s">
         <v>71</v>
       </c>
@@ -17066,8 +17679,11 @@
       <c r="C23" s="33">
         <v>36550</v>
       </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D23">
+        <v>42000</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A24" s="33" t="s">
         <v>72</v>
       </c>
@@ -17077,8 +17693,11 @@
       <c r="C24" s="33">
         <v>38250</v>
       </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D24">
+        <v>48000</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A25" s="33" t="s">
         <v>73</v>
       </c>
@@ -17088,8 +17707,11 @@
       <c r="C25" s="33">
         <v>26350</v>
       </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D25">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A26" s="33" t="s">
         <v>74</v>
       </c>
@@ -17099,8 +17721,11 @@
       <c r="C26" s="33">
         <v>39100</v>
       </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D26">
+        <v>45000</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A27" s="33" t="s">
         <v>75</v>
       </c>
@@ -17110,8 +17735,11 @@
       <c r="C27" s="33">
         <v>36550</v>
       </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D27">
+        <v>46000</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A28" s="33" t="s">
         <v>76</v>
       </c>
@@ -17121,8 +17749,11 @@
       <c r="C28" s="33">
         <v>49300</v>
       </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D28">
+        <v>63000</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A29" s="33" t="s">
         <v>77</v>
       </c>

</xml_diff>